<commit_message>
feat: add marquee feature on homepage and enhance service cards layout
- Implemented a marquee effect for featured items on the homepage.
- Adjusted service cards to include images and improved accessibility features.
- Added a spotlight stage section with image previews and navigation controls.
- Included new SVG icons for navigation in the spotlight section.
</commit_message>
<xml_diff>
--- a/Documentation Planning/pricing.xlsx
+++ b/Documentation Planning/pricing.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\BAGUS BATRA\BB-Photography\Documentation Planning\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BCAA5CF-2EB8-415C-8F2D-972FD141243C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF6EDCF2-2DAF-4278-B0A3-E46D32C7F6B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MENU" sheetId="1" r:id="rId1"/>
-    <sheet name="GRADUATION" sheetId="2" r:id="rId2"/>
-    <sheet name="COUPLE" sheetId="3" r:id="rId3"/>
-    <sheet name="PERSONAL" sheetId="4" r:id="rId4"/>
-    <sheet name="BEAUTY" sheetId="5" r:id="rId5"/>
+    <sheet name="PERSONAL" sheetId="4" r:id="rId2"/>
+    <sheet name="BEAUTY" sheetId="5" r:id="rId3"/>
+    <sheet name="GRADUATION" sheetId="2" r:id="rId4"/>
+    <sheet name="COUPLE" sheetId="3" r:id="rId5"/>
     <sheet name="PREWEDDING" sheetId="6" r:id="rId6"/>
     <sheet name="WEDDING" sheetId="7" r:id="rId7"/>
     <sheet name="ENGAGEMENT" sheetId="8" r:id="rId8"/>
@@ -27,7 +27,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="5" r:id="rId12"/>
+    <pivotCache cacheId="0" r:id="rId12"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -427,9 +427,9 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -549,16 +549,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
@@ -566,6 +560,12 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -3315,7 +3315,7 @@
     <cacheField name="Client" numFmtId="0">
       <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="4" maxValue="4"/>
     </cacheField>
-    <cacheField name="Stage 1" numFmtId="165">
+    <cacheField name="Stage 1" numFmtId="164">
       <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="700000" maxValue="5200000" count="9">
         <n v="860000"/>
         <n v="940000"/>
@@ -3328,7 +3328,7 @@
         <n v="3360000"/>
       </sharedItems>
     </cacheField>
-    <cacheField name="Stage 2" numFmtId="165">
+    <cacheField name="Stage 2" numFmtId="164">
       <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="1300000" maxValue="9600000" count="6">
         <n v="1300000"/>
         <n v="1900000"/>
@@ -3338,10 +3338,10 @@
         <n v="6160000"/>
       </sharedItems>
     </cacheField>
-    <cacheField name="Stage 3" numFmtId="165">
+    <cacheField name="Stage 3" numFmtId="164">
       <sharedItems containsMixedTypes="1" containsNumber="1" containsInteger="1" minValue="2300000" maxValue="15200000"/>
     </cacheField>
-    <cacheField name="Stage 4" numFmtId="165">
+    <cacheField name="Stage 4" numFmtId="164">
       <sharedItems containsMixedTypes="1" containsNumber="1" containsInteger="1" minValue="3900000" maxValue="32800000"/>
     </cacheField>
   </cacheFields>
@@ -3431,7 +3431,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{76FA9080-9907-4BEB-ACB7-E85178F5C4E7}" name="PivotTable1" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{76FA9080-9907-4BEB-ACB7-E85178F5C4E7}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
   <location ref="B14:F24" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="6">
     <pivotField axis="axisRow" showAll="0">
@@ -3449,7 +3449,7 @@
       </items>
     </pivotField>
     <pivotField showAll="0"/>
-    <pivotField dataField="1" numFmtId="165" showAll="0">
+    <pivotField dataField="1" numFmtId="164" showAll="0">
       <items count="10">
         <item x="3"/>
         <item x="0"/>
@@ -3463,7 +3463,7 @@
         <item t="default"/>
       </items>
     </pivotField>
-    <pivotField dataField="1" numFmtId="165" showAll="0">
+    <pivotField dataField="1" numFmtId="164" showAll="0">
       <items count="7">
         <item x="0"/>
         <item x="1"/>
@@ -4038,7 +4038,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4047,7 +4047,7 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1071EBF4-91EE-4334-B20E-AE85B91A2517}">
   <dimension ref="B1:G34"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="1"/>
     <col min="2" max="2" width="36" style="1" customWidth="1"/>
@@ -4059,36 +4059,36 @@
     <col min="8" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:7" ht="30" customHeight="1"/>
-    <row r="2" spans="2:7" ht="25.5" customHeight="1">
+    <row r="1" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="2:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="5" t="s">
         <v>91</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="F2" s="13" t="s">
+      <c r="F2" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="13"/>
-    </row>
-    <row r="3" spans="2:7" ht="25.5" customHeight="1">
+      <c r="G2" s="18"/>
+    </row>
+    <row r="3" spans="2:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="3">
         <v>840000</v>
       </c>
       <c r="D3" s="3">
         <v>1540000</v>
       </c>
-      <c r="F3" s="13"/>
-      <c r="G3" s="13"/>
-    </row>
-    <row r="4" spans="2:7" ht="6" customHeight="1">
+      <c r="F3" s="18"/>
+      <c r="G3" s="18"/>
+    </row>
+    <row r="4" spans="2:7" ht="6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="4"/>
       <c r="D4" s="4"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
     </row>
-    <row r="5" spans="2:7">
+    <row r="5" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B5" s="4" t="s">
         <v>88</v>
       </c>
@@ -4102,7 +4102,7 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="6" spans="2:7">
+    <row r="6" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B6" s="4" t="s">
         <v>64</v>
       </c>
@@ -4116,7 +4116,7 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="7" spans="2:7">
+    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B7" s="4" t="s">
         <v>65</v>
       </c>
@@ -4130,7 +4130,7 @@
         <v>350000</v>
       </c>
     </row>
-    <row r="8" spans="2:7">
+    <row r="8" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B8" s="4" t="s">
         <v>4</v>
       </c>
@@ -4144,50 +4144,50 @@
         <v>50000</v>
       </c>
     </row>
-    <row r="9" spans="2:7">
+    <row r="9" spans="2:7" x14ac:dyDescent="0.25">
       <c r="D9" s="4" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="10" spans="2:7">
+    <row r="10" spans="2:7" x14ac:dyDescent="0.25">
       <c r="D10" s="4" t="s">
         <v>4</v>
       </c>
       <c r="F10" s="10"/>
       <c r="G10" s="11"/>
     </row>
-    <row r="12" spans="2:7">
+    <row r="12" spans="2:7" x14ac:dyDescent="0.25">
       <c r="D12" s="10"/>
     </row>
-    <row r="14" spans="2:7" ht="26.25" customHeight="1">
+    <row r="14" spans="2:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="5" t="s">
         <v>92</v>
       </c>
       <c r="D14" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="F14" s="14" t="s">
+      <c r="F14" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="G14" s="13"/>
-    </row>
-    <row r="15" spans="2:7" ht="25.5" customHeight="1">
+      <c r="G14" s="18"/>
+    </row>
+    <row r="15" spans="2:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="3">
         <v>2800000</v>
       </c>
       <c r="D15" s="3">
         <v>5400000</v>
       </c>
-      <c r="F15" s="13"/>
-      <c r="G15" s="13"/>
-    </row>
-    <row r="16" spans="2:7" ht="6.75" customHeight="1">
+      <c r="F15" s="18"/>
+      <c r="G15" s="18"/>
+    </row>
+    <row r="16" spans="2:7" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="4"/>
       <c r="D16" s="4"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
     </row>
-    <row r="17" spans="2:7">
+    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B17" s="4" t="s">
         <v>90</v>
       </c>
@@ -4201,7 +4201,7 @@
         <v>-50000</v>
       </c>
     </row>
-    <row r="18" spans="2:7">
+    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B18" s="4" t="s">
         <v>64</v>
       </c>
@@ -4216,7 +4216,7 @@
         <v>-50000 &amp; -25000</v>
       </c>
     </row>
-    <row r="19" spans="2:7">
+    <row r="19" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B19" s="4" t="s">
         <v>57</v>
       </c>
@@ -4231,7 +4231,7 @@
         <v>-50% All Type</v>
       </c>
     </row>
-    <row r="20" spans="2:7">
+    <row r="20" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B20" s="4" t="s">
         <v>48</v>
       </c>
@@ -4246,7 +4246,7 @@
         <v>-30% All Type</v>
       </c>
     </row>
-    <row r="21" spans="2:7">
+    <row r="21" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B21" s="4" t="s">
         <v>58</v>
       </c>
@@ -4254,7 +4254,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="22" spans="2:7">
+    <row r="22" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B22" s="4" t="s">
         <v>66</v>
       </c>
@@ -4262,7 +4262,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="23" spans="2:7">
+    <row r="23" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B23" s="4" t="s">
         <v>4</v>
       </c>
@@ -4270,14 +4270,14 @@
         <v>66</v>
       </c>
     </row>
-    <row r="24" spans="2:7">
+    <row r="24" spans="2:7" x14ac:dyDescent="0.25">
       <c r="D24" s="4" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="25" spans="2:7" ht="15.75" customHeight="1"/>
-    <row r="26" spans="2:7" ht="15.75" customHeight="1"/>
-    <row r="34" spans="2:2">
+    <row r="25" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="26" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="34" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B34" s="12"/>
     </row>
   </sheetData>
@@ -4293,7 +4293,7 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2ED714A2-7F80-46E3-BC42-5E655D5C93B7}">
   <dimension ref="B2:U42"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="1"/>
     <col min="2" max="2" width="13.140625" style="1" bestFit="1" customWidth="1"/>
@@ -4303,51 +4303,51 @@
     <col min="22" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:21">
-      <c r="B2" s="15" t="s">
+    <row r="2" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B2" s="13" t="s">
         <v>96</v>
       </c>
-      <c r="C2" s="15" t="s">
+      <c r="C2" s="13" t="s">
         <v>102</v>
       </c>
-      <c r="D2" s="15" t="s">
+      <c r="D2" s="13" t="s">
         <v>98</v>
       </c>
-      <c r="E2" s="15" t="s">
+      <c r="E2" s="13" t="s">
         <v>99</v>
       </c>
-      <c r="F2" s="15" t="s">
+      <c r="F2" s="13" t="s">
         <v>100</v>
       </c>
-      <c r="G2" s="15" t="s">
+      <c r="G2" s="13" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="3" spans="2:21">
+    <row r="3" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B3" s="4" t="s">
         <v>97</v>
       </c>
       <c r="C3" s="4">
         <v>4</v>
       </c>
-      <c r="D3" s="16">
+      <c r="D3" s="14">
         <f>C3*GRADUATION!B3</f>
         <v>860000</v>
       </c>
-      <c r="E3" s="16">
+      <c r="E3" s="14">
         <f>C3*GRADUATION!D3</f>
         <v>1300000</v>
       </c>
-      <c r="F3" s="16">
+      <c r="F3" s="14">
         <f>C3*GRADUATION!B14</f>
         <v>2300000</v>
       </c>
-      <c r="G3" s="16">
+      <c r="G3" s="14">
         <f>4*GRADUATION!D14</f>
         <v>3900000</v>
       </c>
     </row>
-    <row r="4" spans="2:21">
+    <row r="4" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B4" s="4" t="s">
         <v>103</v>
       </c>
@@ -4355,23 +4355,23 @@
         <f>$C$3</f>
         <v>4</v>
       </c>
-      <c r="D4" s="16">
+      <c r="D4" s="14">
         <f>C4*COUPLE!B3</f>
         <v>940000</v>
       </c>
-      <c r="E4" s="16">
+      <c r="E4" s="14">
         <f>C4*COUPLE!D3</f>
         <v>1300000</v>
       </c>
-      <c r="F4" s="16">
+      <c r="F4" s="14">
         <f>C4*COUPLE!B14</f>
         <v>2460000</v>
       </c>
-      <c r="G4" s="16" t="s">
+      <c r="G4" s="14" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="5" spans="2:21">
+    <row r="5" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B5" s="4" t="s">
         <v>104</v>
       </c>
@@ -4379,23 +4379,23 @@
         <f t="shared" ref="C5:C11" si="0">$C$3</f>
         <v>4</v>
       </c>
-      <c r="D5" s="16">
+      <c r="D5" s="14">
         <f>C5*PERSONAL!B3</f>
         <v>900000</v>
       </c>
-      <c r="E5" s="16">
+      <c r="E5" s="14">
         <f>C5*PERSONAL!D3</f>
         <v>1900000</v>
       </c>
-      <c r="F5" s="16">
+      <c r="F5" s="14">
         <f>C5*PERSONAL!B14</f>
         <v>3660000</v>
       </c>
-      <c r="G5" s="16" t="s">
+      <c r="G5" s="14" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="6" spans="2:21">
+    <row r="6" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B6" s="4" t="s">
         <v>105</v>
       </c>
@@ -4403,22 +4403,22 @@
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="D6" s="16">
+      <c r="D6" s="14">
         <f>C6*BEAUTY!B3</f>
         <v>700000</v>
       </c>
-      <c r="E6" s="16">
+      <c r="E6" s="14">
         <f>BEAUTY!D3*C6</f>
         <v>1900000</v>
       </c>
-      <c r="F6" s="16" t="s">
+      <c r="F6" s="14" t="s">
         <v>111</v>
       </c>
-      <c r="G6" s="16" t="s">
+      <c r="G6" s="14" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="7" spans="2:21">
+    <row r="7" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B7" s="4" t="s">
         <v>106</v>
       </c>
@@ -4426,24 +4426,24 @@
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="D7" s="16">
+      <c r="D7" s="14">
         <f>C7*PREWEDDING!B3</f>
         <v>1940000</v>
       </c>
-      <c r="E7" s="16">
+      <c r="E7" s="14">
         <f>C7*PREWEDDING!D3</f>
         <v>3800000</v>
       </c>
-      <c r="F7" s="16">
+      <c r="F7" s="14">
         <f>C7*PREWEDDING!B15</f>
         <v>7200000</v>
       </c>
-      <c r="G7" s="16">
+      <c r="G7" s="14">
         <f>C7*PREWEDDING!D15</f>
         <v>15200000</v>
       </c>
     </row>
-    <row r="8" spans="2:21">
+    <row r="8" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B8" s="4" t="s">
         <v>107</v>
       </c>
@@ -4451,24 +4451,24 @@
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="D8" s="16">
+      <c r="D8" s="14">
         <f>C8*WEDDING!B3</f>
         <v>5200000</v>
       </c>
-      <c r="E8" s="16">
+      <c r="E8" s="14">
         <f>C8*WEDDING!D3</f>
         <v>9600000</v>
       </c>
-      <c r="F8" s="16">
+      <c r="F8" s="14">
         <f>C8*WEDDING!B15</f>
         <v>15200000</v>
       </c>
-      <c r="G8" s="16">
+      <c r="G8" s="14">
         <f>C8*WEDDING!D15</f>
         <v>32800000</v>
       </c>
     </row>
-    <row r="9" spans="2:21">
+    <row r="9" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B9" s="4" t="s">
         <v>108</v>
       </c>
@@ -4476,24 +4476,24 @@
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="D9" s="16">
+      <c r="D9" s="14">
         <f>C9*ENGAGEMENT!B3</f>
         <v>2200000</v>
       </c>
-      <c r="E9" s="16">
+      <c r="E9" s="14">
         <f>C9*ENGAGEMENT!D3</f>
         <v>3680000</v>
       </c>
-      <c r="F9" s="16">
+      <c r="F9" s="14">
         <f>C9*ENGAGEMENT!B15</f>
         <v>6400000</v>
       </c>
-      <c r="G9" s="16">
+      <c r="G9" s="14">
         <f>C9*ENGAGEMENT!D15</f>
         <v>19200000</v>
       </c>
     </row>
-    <row r="10" spans="2:21">
+    <row r="10" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B10" s="4" t="s">
         <v>109</v>
       </c>
@@ -4501,24 +4501,24 @@
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="D10" s="16">
+      <c r="D10" s="14">
         <f>C10*EVENT!B3</f>
         <v>2080000</v>
       </c>
-      <c r="E10" s="16">
+      <c r="E10" s="14">
         <f>C10*EVENT!D3</f>
         <v>3680000</v>
       </c>
-      <c r="F10" s="16">
+      <c r="F10" s="14">
         <f>C10*EVENT!B15</f>
         <v>6400000</v>
       </c>
-      <c r="G10" s="16">
+      <c r="G10" s="14">
         <f>C10*EVENT!D15</f>
         <v>19200000</v>
       </c>
     </row>
-    <row r="11" spans="2:21">
+    <row r="11" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B11" s="4" t="s">
         <v>110</v>
       </c>
@@ -4526,25 +4526,25 @@
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="D11" s="16">
+      <c r="D11" s="14">
         <f>C11*TRAVEL!B3</f>
         <v>3360000</v>
       </c>
-      <c r="E11" s="16">
+      <c r="E11" s="14">
         <f>C11*TRAVEL!D3</f>
         <v>6160000</v>
       </c>
-      <c r="F11" s="16">
+      <c r="F11" s="14">
         <f>C11*TRAVEL!B15</f>
         <v>11200000</v>
       </c>
-      <c r="G11" s="16">
+      <c r="G11" s="14">
         <f>C11*TRAVEL!D15</f>
         <v>21600000</v>
       </c>
     </row>
-    <row r="14" spans="2:21">
-      <c r="B14" s="17" t="s">
+    <row r="14" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B14" s="15" t="s">
         <v>113</v>
       </c>
       <c r="C14" t="s">
@@ -4575,20 +4575,20 @@
       <c r="T14"/>
       <c r="U14"/>
     </row>
-    <row r="15" spans="2:21">
-      <c r="B15" s="18" t="s">
+    <row r="15" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B15" s="16" t="s">
         <v>105</v>
       </c>
-      <c r="C15" s="19">
+      <c r="C15" s="17">
         <v>700000</v>
       </c>
-      <c r="D15" s="19">
+      <c r="D15" s="17">
         <v>1900000</v>
       </c>
-      <c r="E15" s="19">
+      <c r="E15" s="17">
         <v>0</v>
       </c>
-      <c r="F15" s="19">
+      <c r="F15" s="17">
         <v>0</v>
       </c>
       <c r="G15"/>
@@ -4607,20 +4607,20 @@
       <c r="T15"/>
       <c r="U15"/>
     </row>
-    <row r="16" spans="2:21">
-      <c r="B16" s="18" t="s">
+    <row r="16" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B16" s="16" t="s">
         <v>103</v>
       </c>
-      <c r="C16" s="19">
+      <c r="C16" s="17">
         <v>940000</v>
       </c>
-      <c r="D16" s="19">
+      <c r="D16" s="17">
         <v>1300000</v>
       </c>
-      <c r="E16" s="19">
+      <c r="E16" s="17">
         <v>2460000</v>
       </c>
-      <c r="F16" s="19">
+      <c r="F16" s="17">
         <v>0</v>
       </c>
       <c r="G16"/>
@@ -4639,20 +4639,20 @@
       <c r="T16"/>
       <c r="U16"/>
     </row>
-    <row r="17" spans="2:21">
-      <c r="B17" s="18" t="s">
+    <row r="17" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B17" s="16" t="s">
         <v>108</v>
       </c>
-      <c r="C17" s="19">
+      <c r="C17" s="17">
         <v>2200000</v>
       </c>
-      <c r="D17" s="19">
+      <c r="D17" s="17">
         <v>3680000</v>
       </c>
-      <c r="E17" s="19">
+      <c r="E17" s="17">
         <v>6400000</v>
       </c>
-      <c r="F17" s="19">
+      <c r="F17" s="17">
         <v>19200000</v>
       </c>
       <c r="G17"/>
@@ -4671,20 +4671,20 @@
       <c r="T17"/>
       <c r="U17"/>
     </row>
-    <row r="18" spans="2:21">
-      <c r="B18" s="18" t="s">
+    <row r="18" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B18" s="16" t="s">
         <v>109</v>
       </c>
-      <c r="C18" s="19">
+      <c r="C18" s="17">
         <v>2080000</v>
       </c>
-      <c r="D18" s="19">
+      <c r="D18" s="17">
         <v>3680000</v>
       </c>
-      <c r="E18" s="19">
+      <c r="E18" s="17">
         <v>6400000</v>
       </c>
-      <c r="F18" s="19">
+      <c r="F18" s="17">
         <v>19200000</v>
       </c>
       <c r="G18"/>
@@ -4703,20 +4703,20 @@
       <c r="T18"/>
       <c r="U18"/>
     </row>
-    <row r="19" spans="2:21">
-      <c r="B19" s="18" t="s">
+    <row r="19" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B19" s="16" t="s">
         <v>97</v>
       </c>
-      <c r="C19" s="19">
+      <c r="C19" s="17">
         <v>860000</v>
       </c>
-      <c r="D19" s="19">
+      <c r="D19" s="17">
         <v>1300000</v>
       </c>
-      <c r="E19" s="19">
+      <c r="E19" s="17">
         <v>2300000</v>
       </c>
-      <c r="F19" s="19">
+      <c r="F19" s="17">
         <v>3900000</v>
       </c>
       <c r="G19"/>
@@ -4735,20 +4735,20 @@
       <c r="T19"/>
       <c r="U19"/>
     </row>
-    <row r="20" spans="2:21">
-      <c r="B20" s="18" t="s">
+    <row r="20" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B20" s="16" t="s">
         <v>104</v>
       </c>
-      <c r="C20" s="19">
+      <c r="C20" s="17">
         <v>900000</v>
       </c>
-      <c r="D20" s="19">
+      <c r="D20" s="17">
         <v>1900000</v>
       </c>
-      <c r="E20" s="19">
+      <c r="E20" s="17">
         <v>3660000</v>
       </c>
-      <c r="F20" s="19">
+      <c r="F20" s="17">
         <v>0</v>
       </c>
       <c r="G20"/>
@@ -4767,20 +4767,20 @@
       <c r="T20"/>
       <c r="U20"/>
     </row>
-    <row r="21" spans="2:21">
-      <c r="B21" s="18" t="s">
+    <row r="21" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B21" s="16" t="s">
         <v>106</v>
       </c>
-      <c r="C21" s="19">
+      <c r="C21" s="17">
         <v>1940000</v>
       </c>
-      <c r="D21" s="19">
+      <c r="D21" s="17">
         <v>3800000</v>
       </c>
-      <c r="E21" s="19">
+      <c r="E21" s="17">
         <v>7200000</v>
       </c>
-      <c r="F21" s="19">
+      <c r="F21" s="17">
         <v>15200000</v>
       </c>
       <c r="G21"/>
@@ -4799,20 +4799,20 @@
       <c r="T21"/>
       <c r="U21"/>
     </row>
-    <row r="22" spans="2:21">
-      <c r="B22" s="18" t="s">
+    <row r="22" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B22" s="16" t="s">
         <v>110</v>
       </c>
-      <c r="C22" s="19">
+      <c r="C22" s="17">
         <v>3360000</v>
       </c>
-      <c r="D22" s="19">
+      <c r="D22" s="17">
         <v>6160000</v>
       </c>
-      <c r="E22" s="19">
+      <c r="E22" s="17">
         <v>11200000</v>
       </c>
-      <c r="F22" s="19">
+      <c r="F22" s="17">
         <v>21600000</v>
       </c>
       <c r="G22"/>
@@ -4831,20 +4831,20 @@
       <c r="T22"/>
       <c r="U22"/>
     </row>
-    <row r="23" spans="2:21">
-      <c r="B23" s="18" t="s">
+    <row r="23" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B23" s="16" t="s">
         <v>107</v>
       </c>
-      <c r="C23" s="19">
+      <c r="C23" s="17">
         <v>5200000</v>
       </c>
-      <c r="D23" s="19">
+      <c r="D23" s="17">
         <v>9600000</v>
       </c>
-      <c r="E23" s="19">
+      <c r="E23" s="17">
         <v>15200000</v>
       </c>
-      <c r="F23" s="19">
+      <c r="F23" s="17">
         <v>32800000</v>
       </c>
       <c r="G23"/>
@@ -4863,20 +4863,20 @@
       <c r="T23"/>
       <c r="U23"/>
     </row>
-    <row r="24" spans="2:21">
-      <c r="B24" s="18" t="s">
+    <row r="24" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="B24" s="16" t="s">
         <v>112</v>
       </c>
-      <c r="C24" s="19">
+      <c r="C24" s="17">
         <v>18180000</v>
       </c>
-      <c r="D24" s="19">
+      <c r="D24" s="17">
         <v>33320000</v>
       </c>
-      <c r="E24" s="19">
+      <c r="E24" s="17">
         <v>54820000</v>
       </c>
-      <c r="F24" s="19">
+      <c r="F24" s="17">
         <v>111900000</v>
       </c>
       <c r="G24"/>
@@ -4895,7 +4895,7 @@
       <c r="T24"/>
       <c r="U24"/>
     </row>
-    <row r="25" spans="2:21">
+    <row r="25" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B25"/>
       <c r="C25"/>
       <c r="D25"/>
@@ -4917,7 +4917,7 @@
       <c r="T25"/>
       <c r="U25"/>
     </row>
-    <row r="26" spans="2:21">
+    <row r="26" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B26"/>
       <c r="C26"/>
       <c r="D26"/>
@@ -4939,7 +4939,7 @@
       <c r="T26"/>
       <c r="U26"/>
     </row>
-    <row r="27" spans="2:21">
+    <row r="27" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B27"/>
       <c r="C27"/>
       <c r="D27"/>
@@ -4952,7 +4952,7 @@
       <c r="K27"/>
       <c r="L27"/>
     </row>
-    <row r="28" spans="2:21">
+    <row r="28" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B28"/>
       <c r="C28"/>
       <c r="D28"/>
@@ -4965,7 +4965,7 @@
       <c r="K28"/>
       <c r="L28"/>
     </row>
-    <row r="29" spans="2:21">
+    <row r="29" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B29"/>
       <c r="C29"/>
       <c r="D29"/>
@@ -4978,7 +4978,7 @@
       <c r="K29"/>
       <c r="L29"/>
     </row>
-    <row r="30" spans="2:21">
+    <row r="30" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B30"/>
       <c r="C30"/>
       <c r="D30"/>
@@ -4991,7 +4991,7 @@
       <c r="K30"/>
       <c r="L30"/>
     </row>
-    <row r="31" spans="2:21">
+    <row r="31" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B31"/>
       <c r="C31"/>
       <c r="D31"/>
@@ -5004,7 +5004,7 @@
       <c r="K31"/>
       <c r="L31"/>
     </row>
-    <row r="32" spans="2:21">
+    <row r="32" spans="2:21" x14ac:dyDescent="0.25">
       <c r="B32"/>
       <c r="C32"/>
       <c r="D32"/>
@@ -5017,7 +5017,7 @@
       <c r="K32"/>
       <c r="L32"/>
     </row>
-    <row r="33" spans="2:12">
+    <row r="33" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B33"/>
       <c r="C33"/>
       <c r="D33"/>
@@ -5030,7 +5030,7 @@
       <c r="K33"/>
       <c r="L33"/>
     </row>
-    <row r="34" spans="2:12">
+    <row r="34" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B34"/>
       <c r="C34"/>
       <c r="D34"/>
@@ -5043,28 +5043,28 @@
       <c r="K34"/>
       <c r="L34"/>
     </row>
-    <row r="35" spans="2:12">
+    <row r="35" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B35"/>
     </row>
-    <row r="36" spans="2:12">
+    <row r="36" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B36"/>
     </row>
-    <row r="37" spans="2:12">
+    <row r="37" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B37"/>
     </row>
-    <row r="38" spans="2:12">
+    <row r="38" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B38"/>
     </row>
-    <row r="39" spans="2:12">
+    <row r="39" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B39"/>
     </row>
-    <row r="40" spans="2:12">
+    <row r="40" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B40"/>
     </row>
-    <row r="41" spans="2:12">
+    <row r="41" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B41"/>
     </row>
-    <row r="42" spans="2:12">
+    <row r="42" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B42"/>
     </row>
   </sheetData>
@@ -5074,9 +5074,9 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9BA0498E-CFF0-4389-A69A-34CB8E5E601C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F09C4C1-1C9C-429F-AA75-8EBC75D29B6C}">
   <dimension ref="B1:G25"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="1"/>
     <col min="2" max="2" width="36" style="1" customWidth="1"/>
@@ -5088,41 +5088,41 @@
     <col min="8" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:7" ht="30" customHeight="1"/>
-    <row r="2" spans="2:7" ht="25.5" customHeight="1">
+    <row r="1" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="2:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="2" t="s">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="F2" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="F2" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="13"/>
-    </row>
-    <row r="3" spans="2:7" ht="25.5" customHeight="1">
+      <c r="G2" s="18"/>
+    </row>
+    <row r="3" spans="2:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="3">
-        <v>215000</v>
+        <v>225000</v>
       </c>
       <c r="D3" s="3">
-        <v>325000</v>
-      </c>
-      <c r="F3" s="13"/>
-      <c r="G3" s="13"/>
-    </row>
-    <row r="4" spans="2:7" ht="6" customHeight="1">
+        <v>475000</v>
+      </c>
+      <c r="F3" s="18"/>
+      <c r="G3" s="18"/>
+    </row>
+    <row r="4" spans="2:7" ht="6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="4"/>
       <c r="D4" s="4"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
     </row>
-    <row r="5" spans="2:7">
+    <row r="5" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B5" s="4" t="s">
         <v>2</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="F5" s="4" t="s">
         <v>17</v>
@@ -5131,12 +5131,12 @@
         <v>80000</v>
       </c>
     </row>
-    <row r="6" spans="2:7">
+    <row r="6" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B6" s="4" t="s">
         <v>1</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F6" s="4" t="s">
         <v>1</v>
@@ -5145,7 +5145,7 @@
         <v>100000</v>
       </c>
     </row>
-    <row r="7" spans="2:7">
+    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B7" s="4" t="s">
         <v>3</v>
       </c>
@@ -5159,7 +5159,7 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="8" spans="2:7">
+    <row r="8" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B8" s="4" t="s">
         <v>4</v>
       </c>
@@ -5173,7 +5173,7 @@
         <v>35000</v>
       </c>
     </row>
-    <row r="9" spans="2:7">
+    <row r="9" spans="2:7" x14ac:dyDescent="0.25">
       <c r="D9" s="4" t="s">
         <v>7</v>
       </c>
@@ -5184,41 +5184,40 @@
         <v>50000</v>
       </c>
     </row>
-    <row r="13" spans="2:7" ht="26.25" customHeight="1">
+    <row r="10" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="D10" s="4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="13" spans="2:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F13" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="D13" s="8"/>
+      <c r="F13" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="G13" s="13"/>
-    </row>
-    <row r="14" spans="2:7" ht="25.5" customHeight="1">
+      <c r="G13" s="18"/>
+    </row>
+    <row r="14" spans="2:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="3">
-        <v>575000</v>
-      </c>
-      <c r="D14" s="3">
-        <v>975000</v>
-      </c>
-      <c r="F14" s="13"/>
-      <c r="G14" s="13"/>
-    </row>
-    <row r="15" spans="2:7" ht="6.75" customHeight="1">
+        <v>915000</v>
+      </c>
+      <c r="D14" s="9"/>
+      <c r="F14" s="18"/>
+      <c r="G14" s="18"/>
+    </row>
+    <row r="15" spans="2:7" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="4"/>
-      <c r="D15" s="4"/>
+      <c r="D15" s="10"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
     </row>
-    <row r="16" spans="2:7">
+    <row r="16" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B16" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D16" s="4" t="s">
-        <v>14</v>
-      </c>
+      <c r="D16" s="10"/>
       <c r="F16" s="4" t="s">
         <v>20</v>
       </c>
@@ -5226,13 +5225,11 @@
         <v>-50000</v>
       </c>
     </row>
-    <row r="17" spans="2:7">
+    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B17" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>13</v>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="D17" s="10"/>
       <c r="F17" s="4" t="s">
         <v>21</v>
       </c>
@@ -5241,13 +5238,11 @@
         <v>-50000 &amp; -25000</v>
       </c>
     </row>
-    <row r="18" spans="2:7">
+    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B18" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D18" s="4" t="s">
-        <v>11</v>
-      </c>
+      <c r="D18" s="10"/>
       <c r="F18" s="4" t="s">
         <v>22</v>
       </c>
@@ -5256,31 +5251,30 @@
         <v>-50% All Type</v>
       </c>
     </row>
-    <row r="19" spans="2:7">
+    <row r="19" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B19" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D19" s="4" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="20" spans="2:7">
+      <c r="D19" s="10"/>
+    </row>
+    <row r="20" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B20" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D20" s="4" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="21" spans="2:7">
+      <c r="D20" s="10"/>
+    </row>
+    <row r="21" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B21" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D21" s="4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="25" spans="2:7" ht="26.25" customHeight="1"/>
+        <v>33</v>
+      </c>
+      <c r="D21" s="10"/>
+    </row>
+    <row r="22" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B22" s="4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="25" spans="2:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="F2:G3"/>
@@ -5292,9 +5286,9 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4510C927-4F2F-4896-BBDB-E8861F8EED92}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3624BA3E-0F1D-4DE8-8401-F1BA58FC44F6}">
   <dimension ref="B1:G25"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="1"/>
     <col min="2" max="2" width="36" style="1" customWidth="1"/>
@@ -5306,41 +5300,41 @@
     <col min="8" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:7" ht="30" customHeight="1"/>
-    <row r="2" spans="2:7" ht="25.5" customHeight="1">
+    <row r="1" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="2:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="2" t="s">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="F2" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="F2" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="13"/>
-    </row>
-    <row r="3" spans="2:7" ht="25.5" customHeight="1">
+      <c r="G2" s="18"/>
+    </row>
+    <row r="3" spans="2:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="3">
-        <v>235000</v>
+        <v>175000</v>
       </c>
       <c r="D3" s="3">
-        <v>325000</v>
-      </c>
-      <c r="F3" s="13"/>
-      <c r="G3" s="13"/>
-    </row>
-    <row r="4" spans="2:7" ht="6" customHeight="1">
+        <v>475000</v>
+      </c>
+      <c r="F3" s="18"/>
+      <c r="G3" s="18"/>
+    </row>
+    <row r="4" spans="2:7" ht="6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="4"/>
       <c r="D4" s="4"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
     </row>
-    <row r="5" spans="2:7">
+    <row r="5" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B5" s="4" t="s">
         <v>2</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="F5" s="4" t="s">
         <v>17</v>
@@ -5349,12 +5343,12 @@
         <v>80000</v>
       </c>
     </row>
-    <row r="6" spans="2:7">
+    <row r="6" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B6" s="4" t="s">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="F6" s="4" t="s">
         <v>1</v>
@@ -5363,12 +5357,12 @@
         <v>100000</v>
       </c>
     </row>
-    <row r="7" spans="2:7">
+    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B7" s="4" t="s">
         <v>3</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>3</v>
+        <v>38</v>
       </c>
       <c r="F7" s="4" t="s">
         <v>18</v>
@@ -5377,12 +5371,12 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="8" spans="2:7">
+    <row r="8" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B8" s="4" t="s">
         <v>4</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="F8" s="4" t="s">
         <v>3</v>
@@ -5391,9 +5385,9 @@
         <v>35000</v>
       </c>
     </row>
-    <row r="9" spans="2:7">
+    <row r="9" spans="2:7" x14ac:dyDescent="0.25">
       <c r="D9" s="4" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="F9" s="4" t="s">
         <v>19</v>
@@ -5402,34 +5396,38 @@
         <v>50000</v>
       </c>
     </row>
-    <row r="13" spans="2:7" ht="26.25" customHeight="1">
-      <c r="B13" s="2" t="s">
-        <v>27</v>
-      </c>
+    <row r="10" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="D10" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="D11" s="4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="13" spans="2:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="8"/>
       <c r="D13" s="8"/>
-      <c r="F13" s="14" t="s">
+      <c r="F13" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="G13" s="13"/>
-    </row>
-    <row r="14" spans="2:7" ht="25.5" customHeight="1">
-      <c r="B14" s="3">
-        <v>615000</v>
-      </c>
+      <c r="G13" s="18"/>
+    </row>
+    <row r="14" spans="2:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="9"/>
       <c r="D14" s="9"/>
-      <c r="F14" s="13"/>
-      <c r="G14" s="13"/>
-    </row>
-    <row r="15" spans="2:7" ht="6.75" customHeight="1">
-      <c r="B15" s="4"/>
+      <c r="F14" s="18"/>
+      <c r="G14" s="18"/>
+    </row>
+    <row r="15" spans="2:7" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="10"/>
       <c r="D15" s="10"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
     </row>
-    <row r="16" spans="2:7">
-      <c r="B16" s="4" t="s">
-        <v>9</v>
-      </c>
+    <row r="16" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B16" s="10"/>
       <c r="D16" s="10"/>
       <c r="F16" s="4" t="s">
         <v>20</v>
@@ -5438,10 +5436,8 @@
         <v>-50000</v>
       </c>
     </row>
-    <row r="17" spans="2:7">
-      <c r="B17" s="4" t="s">
-        <v>28</v>
-      </c>
+    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B17" s="10"/>
       <c r="D17" s="10"/>
       <c r="F17" s="4" t="s">
         <v>21</v>
@@ -5451,10 +5447,8 @@
         <v>-50000 &amp; -25000</v>
       </c>
     </row>
-    <row r="18" spans="2:7">
-      <c r="B18" s="4" t="s">
-        <v>11</v>
-      </c>
+    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B18" s="10"/>
       <c r="D18" s="10"/>
       <c r="F18" s="4" t="s">
         <v>22</v>
@@ -5464,30 +5458,22 @@
         <v>-50% All Type</v>
       </c>
     </row>
-    <row r="19" spans="2:7">
-      <c r="B19" s="4" t="s">
-        <v>4</v>
-      </c>
+    <row r="19" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B19" s="10"/>
       <c r="D19" s="10"/>
     </row>
-    <row r="20" spans="2:7">
-      <c r="B20" s="4" t="s">
-        <v>7</v>
-      </c>
+    <row r="20" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B20" s="10"/>
       <c r="D20" s="10"/>
     </row>
-    <row r="21" spans="2:7">
-      <c r="B21" s="4" t="s">
-        <v>12</v>
-      </c>
+    <row r="21" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B21" s="10"/>
       <c r="D21" s="10"/>
     </row>
-    <row r="22" spans="2:7">
-      <c r="B22" s="4" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="25" spans="2:7" ht="26.25" customHeight="1"/>
+    <row r="22" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B22" s="10"/>
+    </row>
+    <row r="25" spans="2:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="F2:G3"/>
@@ -5499,9 +5485,9 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F09C4C1-1C9C-429F-AA75-8EBC75D29B6C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9BA0498E-CFF0-4389-A69A-34CB8E5E601C}">
   <dimension ref="B1:G25"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="1"/>
     <col min="2" max="2" width="36" style="1" customWidth="1"/>
@@ -5513,41 +5499,41 @@
     <col min="8" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:7" ht="30" customHeight="1"/>
-    <row r="2" spans="2:7" ht="25.5" customHeight="1">
+    <row r="1" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="2:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="2" t="s">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="F2" s="13" t="s">
+        <v>5</v>
+      </c>
+      <c r="F2" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="13"/>
-    </row>
-    <row r="3" spans="2:7" ht="25.5" customHeight="1">
+      <c r="G2" s="18"/>
+    </row>
+    <row r="3" spans="2:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="3">
-        <v>225000</v>
+        <v>215000</v>
       </c>
       <c r="D3" s="3">
-        <v>475000</v>
-      </c>
-      <c r="F3" s="13"/>
-      <c r="G3" s="13"/>
-    </row>
-    <row r="4" spans="2:7" ht="6" customHeight="1">
+        <v>325000</v>
+      </c>
+      <c r="F3" s="18"/>
+      <c r="G3" s="18"/>
+    </row>
+    <row r="4" spans="2:7" ht="6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="4"/>
       <c r="D4" s="4"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
     </row>
-    <row r="5" spans="2:7">
+    <row r="5" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B5" s="4" t="s">
         <v>2</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="F5" s="4" t="s">
         <v>17</v>
@@ -5556,12 +5542,12 @@
         <v>80000</v>
       </c>
     </row>
-    <row r="6" spans="2:7">
+    <row r="6" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B6" s="4" t="s">
         <v>1</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F6" s="4" t="s">
         <v>1</v>
@@ -5570,7 +5556,7 @@
         <v>100000</v>
       </c>
     </row>
-    <row r="7" spans="2:7">
+    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B7" s="4" t="s">
         <v>3</v>
       </c>
@@ -5584,7 +5570,7 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="8" spans="2:7">
+    <row r="8" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B8" s="4" t="s">
         <v>4</v>
       </c>
@@ -5598,7 +5584,7 @@
         <v>35000</v>
       </c>
     </row>
-    <row r="9" spans="2:7">
+    <row r="9" spans="2:7" x14ac:dyDescent="0.25">
       <c r="D9" s="4" t="s">
         <v>7</v>
       </c>
@@ -5609,40 +5595,41 @@
         <v>50000</v>
       </c>
     </row>
-    <row r="10" spans="2:7">
-      <c r="D10" s="4" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="13" spans="2:7" ht="26.25" customHeight="1">
+    <row r="13" spans="2:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="D13" s="8"/>
-      <c r="F13" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F13" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="G13" s="13"/>
-    </row>
-    <row r="14" spans="2:7" ht="25.5" customHeight="1">
+      <c r="G13" s="18"/>
+    </row>
+    <row r="14" spans="2:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="3">
-        <v>915000</v>
-      </c>
-      <c r="D14" s="9"/>
-      <c r="F14" s="13"/>
-      <c r="G14" s="13"/>
-    </row>
-    <row r="15" spans="2:7" ht="6.75" customHeight="1">
+        <v>575000</v>
+      </c>
+      <c r="D14" s="3">
+        <v>975000</v>
+      </c>
+      <c r="F14" s="18"/>
+      <c r="G14" s="18"/>
+    </row>
+    <row r="15" spans="2:7" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="4"/>
-      <c r="D15" s="10"/>
+      <c r="D15" s="4"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
     </row>
-    <row r="16" spans="2:7">
+    <row r="16" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B16" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D16" s="10"/>
+      <c r="D16" s="4" t="s">
+        <v>14</v>
+      </c>
       <c r="F16" s="4" t="s">
         <v>20</v>
       </c>
@@ -5650,11 +5637,13 @@
         <v>-50000</v>
       </c>
     </row>
-    <row r="17" spans="2:7">
+    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B17" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="D17" s="10"/>
+        <v>10</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>13</v>
+      </c>
       <c r="F17" s="4" t="s">
         <v>21</v>
       </c>
@@ -5663,11 +5652,13 @@
         <v>-50000 &amp; -25000</v>
       </c>
     </row>
-    <row r="18" spans="2:7">
+    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B18" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D18" s="10"/>
+      <c r="D18" s="4" t="s">
+        <v>11</v>
+      </c>
       <c r="F18" s="4" t="s">
         <v>22</v>
       </c>
@@ -5676,30 +5667,31 @@
         <v>-50% All Type</v>
       </c>
     </row>
-    <row r="19" spans="2:7">
+    <row r="19" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B19" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D19" s="10"/>
-    </row>
-    <row r="20" spans="2:7">
+      <c r="D19" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B20" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D20" s="10"/>
-    </row>
-    <row r="21" spans="2:7">
+      <c r="D20" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="21" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B21" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="D21" s="10"/>
-    </row>
-    <row r="22" spans="2:7">
-      <c r="B22" s="4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="25" spans="2:7" ht="26.25" customHeight="1"/>
+        <v>12</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="25" spans="2:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="F2:G3"/>
@@ -5711,9 +5703,9 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3624BA3E-0F1D-4DE8-8401-F1BA58FC44F6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4510C927-4F2F-4896-BBDB-E8861F8EED92}">
   <dimension ref="B1:G25"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="1"/>
     <col min="2" max="2" width="36" style="1" customWidth="1"/>
@@ -5725,41 +5717,41 @@
     <col min="8" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:7" ht="30" customHeight="1"/>
-    <row r="2" spans="2:7" ht="25.5" customHeight="1">
+    <row r="1" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="2:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="2" t="s">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="F2" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="F2" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="13"/>
-    </row>
-    <row r="3" spans="2:7" ht="25.5" customHeight="1">
+      <c r="G2" s="18"/>
+    </row>
+    <row r="3" spans="2:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="3">
-        <v>175000</v>
+        <v>235000</v>
       </c>
       <c r="D3" s="3">
-        <v>475000</v>
-      </c>
-      <c r="F3" s="13"/>
-      <c r="G3" s="13"/>
-    </row>
-    <row r="4" spans="2:7" ht="6" customHeight="1">
+        <v>325000</v>
+      </c>
+      <c r="F3" s="18"/>
+      <c r="G3" s="18"/>
+    </row>
+    <row r="4" spans="2:7" ht="6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="4"/>
       <c r="D4" s="4"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
     </row>
-    <row r="5" spans="2:7">
+    <row r="5" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B5" s="4" t="s">
         <v>2</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="F5" s="4" t="s">
         <v>17</v>
@@ -5768,12 +5760,12 @@
         <v>80000</v>
       </c>
     </row>
-    <row r="6" spans="2:7">
+    <row r="6" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B6" s="4" t="s">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="F6" s="4" t="s">
         <v>1</v>
@@ -5782,12 +5774,12 @@
         <v>100000</v>
       </c>
     </row>
-    <row r="7" spans="2:7">
+    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B7" s="4" t="s">
         <v>3</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>38</v>
+        <v>3</v>
       </c>
       <c r="F7" s="4" t="s">
         <v>18</v>
@@ -5796,12 +5788,12 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="8" spans="2:7">
+    <row r="8" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B8" s="4" t="s">
         <v>4</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="F8" s="4" t="s">
         <v>3</v>
@@ -5810,9 +5802,9 @@
         <v>35000</v>
       </c>
     </row>
-    <row r="9" spans="2:7">
+    <row r="9" spans="2:7" x14ac:dyDescent="0.25">
       <c r="D9" s="4" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="F9" s="4" t="s">
         <v>19</v>
@@ -5821,38 +5813,34 @@
         <v>50000</v>
       </c>
     </row>
-    <row r="10" spans="2:7">
-      <c r="D10" s="4" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="11" spans="2:7">
-      <c r="D11" s="4" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="13" spans="2:7" ht="26.25" customHeight="1">
-      <c r="B13" s="8"/>
+    <row r="13" spans="2:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="D13" s="8"/>
-      <c r="F13" s="14" t="s">
+      <c r="F13" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="G13" s="13"/>
-    </row>
-    <row r="14" spans="2:7" ht="25.5" customHeight="1">
-      <c r="B14" s="9"/>
+      <c r="G13" s="18"/>
+    </row>
+    <row r="14" spans="2:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="3">
+        <v>615000</v>
+      </c>
       <c r="D14" s="9"/>
-      <c r="F14" s="13"/>
-      <c r="G14" s="13"/>
-    </row>
-    <row r="15" spans="2:7" ht="6.75" customHeight="1">
-      <c r="B15" s="10"/>
+      <c r="F14" s="18"/>
+      <c r="G14" s="18"/>
+    </row>
+    <row r="15" spans="2:7" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="4"/>
       <c r="D15" s="10"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
     </row>
-    <row r="16" spans="2:7">
-      <c r="B16" s="10"/>
+    <row r="16" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B16" s="4" t="s">
+        <v>9</v>
+      </c>
       <c r="D16" s="10"/>
       <c r="F16" s="4" t="s">
         <v>20</v>
@@ -5861,8 +5849,10 @@
         <v>-50000</v>
       </c>
     </row>
-    <row r="17" spans="2:7">
-      <c r="B17" s="10"/>
+    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B17" s="4" t="s">
+        <v>28</v>
+      </c>
       <c r="D17" s="10"/>
       <c r="F17" s="4" t="s">
         <v>21</v>
@@ -5872,8 +5862,10 @@
         <v>-50000 &amp; -25000</v>
       </c>
     </row>
-    <row r="18" spans="2:7">
-      <c r="B18" s="10"/>
+    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B18" s="4" t="s">
+        <v>11</v>
+      </c>
       <c r="D18" s="10"/>
       <c r="F18" s="4" t="s">
         <v>22</v>
@@ -5883,22 +5875,30 @@
         <v>-50% All Type</v>
       </c>
     </row>
-    <row r="19" spans="2:7">
-      <c r="B19" s="10"/>
+    <row r="19" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B19" s="4" t="s">
+        <v>4</v>
+      </c>
       <c r="D19" s="10"/>
     </row>
-    <row r="20" spans="2:7">
-      <c r="B20" s="10"/>
+    <row r="20" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B20" s="4" t="s">
+        <v>7</v>
+      </c>
       <c r="D20" s="10"/>
     </row>
-    <row r="21" spans="2:7">
-      <c r="B21" s="10"/>
+    <row r="21" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B21" s="4" t="s">
+        <v>12</v>
+      </c>
       <c r="D21" s="10"/>
     </row>
-    <row r="22" spans="2:7">
-      <c r="B22" s="10"/>
-    </row>
-    <row r="25" spans="2:7" ht="26.25" customHeight="1"/>
+    <row r="22" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B22" s="4" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="25" spans="2:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="F2:G3"/>
@@ -5912,7 +5912,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFE228C7-FCFA-41CE-86C8-CD4AD79C92B0}">
   <dimension ref="B1:G29"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="1"/>
     <col min="2" max="2" width="36" style="1" customWidth="1"/>
@@ -5924,36 +5924,36 @@
     <col min="8" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:7" ht="30" customHeight="1"/>
-    <row r="2" spans="2:7" ht="25.5" customHeight="1">
+    <row r="1" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="2:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="2" t="s">
         <v>39</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="F2" s="13" t="s">
+      <c r="F2" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="13"/>
-    </row>
-    <row r="3" spans="2:7" ht="25.5" customHeight="1">
+      <c r="G2" s="18"/>
+    </row>
+    <row r="3" spans="2:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="3">
         <v>485000</v>
       </c>
       <c r="D3" s="3">
         <v>950000</v>
       </c>
-      <c r="F3" s="13"/>
-      <c r="G3" s="13"/>
-    </row>
-    <row r="4" spans="2:7" ht="6" customHeight="1">
+      <c r="F3" s="18"/>
+      <c r="G3" s="18"/>
+    </row>
+    <row r="4" spans="2:7" ht="6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="4"/>
       <c r="D4" s="4"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
     </row>
-    <row r="5" spans="2:7">
+    <row r="5" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B5" s="4" t="s">
         <v>2</v>
       </c>
@@ -5967,7 +5967,7 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="6" spans="2:7">
+    <row r="6" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B6" s="4" t="s">
         <v>40</v>
       </c>
@@ -5981,7 +5981,7 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="7" spans="2:7">
+    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B7" s="4" t="s">
         <v>41</v>
       </c>
@@ -5995,7 +5995,7 @@
         <v>350000</v>
       </c>
     </row>
-    <row r="8" spans="2:7">
+    <row r="8" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B8" s="4" t="s">
         <v>3</v>
       </c>
@@ -6009,7 +6009,7 @@
         <v>50000</v>
       </c>
     </row>
-    <row r="9" spans="2:7">
+    <row r="9" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B9" s="4" t="s">
         <v>4</v>
       </c>
@@ -6017,50 +6017,50 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="2:7">
+    <row r="10" spans="2:7" x14ac:dyDescent="0.25">
       <c r="D10" s="4" t="s">
         <v>4</v>
       </c>
       <c r="F10" s="10"/>
       <c r="G10" s="11"/>
     </row>
-    <row r="11" spans="2:7">
+    <row r="11" spans="2:7" x14ac:dyDescent="0.25">
       <c r="D11" s="4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="2:7">
+    <row r="12" spans="2:7" x14ac:dyDescent="0.25">
       <c r="D12" s="10"/>
     </row>
-    <row r="14" spans="2:7" ht="26.25" customHeight="1">
+    <row r="14" spans="2:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="2" t="s">
         <v>44</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="F14" s="14" t="s">
+      <c r="F14" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="G14" s="13"/>
-    </row>
-    <row r="15" spans="2:7" ht="25.5" customHeight="1">
+      <c r="G14" s="18"/>
+    </row>
+    <row r="15" spans="2:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="3">
         <v>1800000</v>
       </c>
       <c r="D15" s="3">
         <v>3800000</v>
       </c>
-      <c r="F15" s="13"/>
-      <c r="G15" s="13"/>
-    </row>
-    <row r="16" spans="2:7" ht="6.75" customHeight="1">
+      <c r="F15" s="18"/>
+      <c r="G15" s="18"/>
+    </row>
+    <row r="16" spans="2:7" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="4"/>
       <c r="D16" s="4"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
     </row>
-    <row r="17" spans="2:7">
+    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B17" s="4" t="s">
         <v>45</v>
       </c>
@@ -6074,7 +6074,7 @@
         <v>-50000</v>
       </c>
     </row>
-    <row r="18" spans="2:7">
+    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B18" s="4" t="s">
         <v>40</v>
       </c>
@@ -6089,7 +6089,7 @@
         <v>-50000 &amp; -25000</v>
       </c>
     </row>
-    <row r="19" spans="2:7">
+    <row r="19" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B19" s="4" t="s">
         <v>46</v>
       </c>
@@ -6104,7 +6104,7 @@
         <v>-50% All Type</v>
       </c>
     </row>
-    <row r="20" spans="2:7">
+    <row r="20" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B20" s="4" t="s">
         <v>38</v>
       </c>
@@ -6112,7 +6112,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="21" spans="2:7">
+    <row r="21" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B21" s="4" t="s">
         <v>47</v>
       </c>
@@ -6120,7 +6120,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="22" spans="2:7">
+    <row r="22" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B22" s="4" t="s">
         <v>4</v>
       </c>
@@ -6128,7 +6128,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="23" spans="2:7">
+    <row r="23" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B23" s="4" t="s">
         <v>7</v>
       </c>
@@ -6136,7 +6136,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="24" spans="2:7">
+    <row r="24" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B24" s="4" t="s">
         <v>48</v>
       </c>
@@ -6144,7 +6144,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="25" spans="2:7" ht="15.75" customHeight="1">
+    <row r="25" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="4" t="s">
         <v>49</v>
       </c>
@@ -6152,22 +6152,22 @@
         <v>48</v>
       </c>
     </row>
-    <row r="26" spans="2:7" ht="15.75" customHeight="1">
+    <row r="26" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D26" s="4" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="27" spans="2:7">
+    <row r="27" spans="2:7" x14ac:dyDescent="0.25">
       <c r="D27" s="4" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="28" spans="2:7">
+    <row r="28" spans="2:7" x14ac:dyDescent="0.25">
       <c r="D28" s="4" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="29" spans="2:7">
+    <row r="29" spans="2:7" x14ac:dyDescent="0.25">
       <c r="D29" s="4" t="s">
         <v>59</v>
       </c>
@@ -6185,7 +6185,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C7E75C3-91B2-44EA-9723-79A38490D984}">
   <dimension ref="B1:G28"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="1"/>
     <col min="2" max="2" width="36" style="1" customWidth="1"/>
@@ -6197,36 +6197,36 @@
     <col min="8" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:7" ht="30" customHeight="1"/>
-    <row r="2" spans="2:7" ht="25.5" customHeight="1">
+    <row r="1" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="2:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="2" t="s">
         <v>62</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="F2" s="13" t="s">
+      <c r="F2" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="13"/>
-    </row>
-    <row r="3" spans="2:7" ht="25.5" customHeight="1">
+      <c r="G2" s="18"/>
+    </row>
+    <row r="3" spans="2:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="3">
         <v>1300000</v>
       </c>
       <c r="D3" s="3">
         <v>2400000</v>
       </c>
-      <c r="F3" s="13"/>
-      <c r="G3" s="13"/>
-    </row>
-    <row r="4" spans="2:7" ht="6" customHeight="1">
+      <c r="F3" s="18"/>
+      <c r="G3" s="18"/>
+    </row>
+    <row r="4" spans="2:7" ht="6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="4"/>
       <c r="D4" s="4"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
     </row>
-    <row r="5" spans="2:7">
+    <row r="5" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B5" s="4" t="s">
         <v>63</v>
       </c>
@@ -6240,7 +6240,7 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="6" spans="2:7">
+    <row r="6" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B6" s="4" t="s">
         <v>64</v>
       </c>
@@ -6254,7 +6254,7 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="7" spans="2:7">
+    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B7" s="4" t="s">
         <v>48</v>
       </c>
@@ -6268,7 +6268,7 @@
         <v>350000</v>
       </c>
     </row>
-    <row r="8" spans="2:7">
+    <row r="8" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B8" s="4" t="s">
         <v>65</v>
       </c>
@@ -6282,7 +6282,7 @@
         <v>50000</v>
       </c>
     </row>
-    <row r="9" spans="2:7">
+    <row r="9" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B9" s="4" t="s">
         <v>4</v>
       </c>
@@ -6290,45 +6290,45 @@
         <v>66</v>
       </c>
     </row>
-    <row r="10" spans="2:7">
+    <row r="10" spans="2:7" x14ac:dyDescent="0.25">
       <c r="D10" s="4" t="s">
         <v>4</v>
       </c>
       <c r="F10" s="10"/>
       <c r="G10" s="11"/>
     </row>
-    <row r="12" spans="2:7">
+    <row r="12" spans="2:7" x14ac:dyDescent="0.25">
       <c r="D12" s="10"/>
     </row>
-    <row r="14" spans="2:7" ht="26.25" customHeight="1">
+    <row r="14" spans="2:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="2" t="s">
         <v>71</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="F14" s="14" t="s">
+      <c r="F14" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="G14" s="13"/>
-    </row>
-    <row r="15" spans="2:7" ht="25.5" customHeight="1">
+      <c r="G14" s="18"/>
+    </row>
+    <row r="15" spans="2:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="3">
         <v>3800000</v>
       </c>
       <c r="D15" s="3">
         <v>8200000</v>
       </c>
-      <c r="F15" s="13"/>
-      <c r="G15" s="13"/>
-    </row>
-    <row r="16" spans="2:7" ht="6.75" customHeight="1">
+      <c r="F15" s="18"/>
+      <c r="G15" s="18"/>
+    </row>
+    <row r="16" spans="2:7" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="4"/>
       <c r="D16" s="4"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
     </row>
-    <row r="17" spans="2:7">
+    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B17" s="4" t="s">
         <v>70</v>
       </c>
@@ -6342,7 +6342,7 @@
         <v>-50000</v>
       </c>
     </row>
-    <row r="18" spans="2:7">
+    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B18" s="4" t="s">
         <v>64</v>
       </c>
@@ -6357,7 +6357,7 @@
         <v>-50000 &amp; -25000</v>
       </c>
     </row>
-    <row r="19" spans="2:7">
+    <row r="19" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B19" s="4" t="s">
         <v>57</v>
       </c>
@@ -6372,7 +6372,7 @@
         <v>-50% All Type</v>
       </c>
     </row>
-    <row r="20" spans="2:7">
+    <row r="20" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B20" s="4" t="s">
         <v>69</v>
       </c>
@@ -6380,7 +6380,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="21" spans="2:7">
+    <row r="21" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B21" s="4" t="s">
         <v>58</v>
       </c>
@@ -6388,7 +6388,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="22" spans="2:7">
+    <row r="22" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B22" s="4" t="s">
         <v>66</v>
       </c>
@@ -6396,7 +6396,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="23" spans="2:7">
+    <row r="23" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B23" s="4" t="s">
         <v>4</v>
       </c>
@@ -6404,27 +6404,27 @@
         <v>74</v>
       </c>
     </row>
-    <row r="24" spans="2:7">
+    <row r="24" spans="2:7" x14ac:dyDescent="0.25">
       <c r="D24" s="4" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="25" spans="2:7" ht="15.75" customHeight="1">
+    <row r="25" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D25" s="4" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="26" spans="2:7" ht="15.75" customHeight="1">
+    <row r="26" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D26" s="4" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="27" spans="2:7">
+    <row r="27" spans="2:7" x14ac:dyDescent="0.25">
       <c r="D27" s="4" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="28" spans="2:7">
+    <row r="28" spans="2:7" x14ac:dyDescent="0.25">
       <c r="D28" s="4" t="s">
         <v>59</v>
       </c>
@@ -6442,7 +6442,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{757F7258-105E-4A19-B86D-E5B2236F720D}">
   <dimension ref="B1:G34"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="1"/>
     <col min="2" max="2" width="36" style="1" customWidth="1"/>
@@ -6454,36 +6454,36 @@
     <col min="8" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:7" ht="30" customHeight="1"/>
-    <row r="2" spans="2:7" ht="25.5" customHeight="1">
+    <row r="1" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="2:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="2" t="s">
         <v>84</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="F2" s="13" t="s">
+      <c r="F2" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="13"/>
-    </row>
-    <row r="3" spans="2:7" ht="25.5" customHeight="1">
+      <c r="G2" s="18"/>
+    </row>
+    <row r="3" spans="2:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="3">
         <v>550000</v>
       </c>
       <c r="D3" s="3">
         <v>920000</v>
       </c>
-      <c r="F3" s="13"/>
-      <c r="G3" s="13"/>
-    </row>
-    <row r="4" spans="2:7" ht="6" customHeight="1">
+      <c r="F3" s="18"/>
+      <c r="G3" s="18"/>
+    </row>
+    <row r="4" spans="2:7" ht="6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="4"/>
       <c r="D4" s="4"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
     </row>
-    <row r="5" spans="2:7">
+    <row r="5" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B5" s="4" t="s">
         <v>80</v>
       </c>
@@ -6497,7 +6497,7 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="6" spans="2:7">
+    <row r="6" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B6" s="4" t="s">
         <v>64</v>
       </c>
@@ -6511,7 +6511,7 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="7" spans="2:7">
+    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B7" s="4" t="s">
         <v>48</v>
       </c>
@@ -6525,7 +6525,7 @@
         <v>350000</v>
       </c>
     </row>
-    <row r="8" spans="2:7">
+    <row r="8" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B8" s="4" t="s">
         <v>65</v>
       </c>
@@ -6539,7 +6539,7 @@
         <v>50000</v>
       </c>
     </row>
-    <row r="9" spans="2:7">
+    <row r="9" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B9" s="4" t="s">
         <v>4</v>
       </c>
@@ -6547,45 +6547,45 @@
         <v>66</v>
       </c>
     </row>
-    <row r="10" spans="2:7">
+    <row r="10" spans="2:7" x14ac:dyDescent="0.25">
       <c r="D10" s="4" t="s">
         <v>4</v>
       </c>
       <c r="F10" s="10"/>
       <c r="G10" s="11"/>
     </row>
-    <row r="12" spans="2:7">
+    <row r="12" spans="2:7" x14ac:dyDescent="0.25">
       <c r="D12" s="10"/>
     </row>
-    <row r="14" spans="2:7" ht="26.25" customHeight="1">
+    <row r="14" spans="2:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="2" t="s">
         <v>78</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="F14" s="14" t="s">
+      <c r="F14" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="G14" s="13"/>
-    </row>
-    <row r="15" spans="2:7" ht="25.5" customHeight="1">
+      <c r="G14" s="18"/>
+    </row>
+    <row r="15" spans="2:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="3">
         <v>1600000</v>
       </c>
       <c r="D15" s="3">
         <v>4800000</v>
       </c>
-      <c r="F15" s="13"/>
-      <c r="G15" s="13"/>
-    </row>
-    <row r="16" spans="2:7" ht="6.75" customHeight="1">
+      <c r="F15" s="18"/>
+      <c r="G15" s="18"/>
+    </row>
+    <row r="16" spans="2:7" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="4"/>
       <c r="D16" s="4"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
     </row>
-    <row r="17" spans="2:7">
+    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B17" s="4" t="s">
         <v>81</v>
       </c>
@@ -6599,7 +6599,7 @@
         <v>-50000</v>
       </c>
     </row>
-    <row r="18" spans="2:7">
+    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B18" s="4" t="s">
         <v>64</v>
       </c>
@@ -6614,7 +6614,7 @@
         <v>-50000 &amp; -25000</v>
       </c>
     </row>
-    <row r="19" spans="2:7">
+    <row r="19" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B19" s="4" t="s">
         <v>57</v>
       </c>
@@ -6629,7 +6629,7 @@
         <v>-50% All Type</v>
       </c>
     </row>
-    <row r="20" spans="2:7">
+    <row r="20" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B20" s="4" t="s">
         <v>69</v>
       </c>
@@ -6637,7 +6637,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="21" spans="2:7">
+    <row r="21" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B21" s="4" t="s">
         <v>58</v>
       </c>
@@ -6645,7 +6645,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="22" spans="2:7">
+    <row r="22" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B22" s="4" t="s">
         <v>66</v>
       </c>
@@ -6653,7 +6653,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="23" spans="2:7">
+    <row r="23" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B23" s="4" t="s">
         <v>4</v>
       </c>
@@ -6661,27 +6661,27 @@
         <v>74</v>
       </c>
     </row>
-    <row r="24" spans="2:7">
+    <row r="24" spans="2:7" x14ac:dyDescent="0.25">
       <c r="D24" s="4" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="25" spans="2:7" ht="15.75" customHeight="1">
+    <row r="25" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D25" s="4" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="26" spans="2:7" ht="15.75" customHeight="1">
+    <row r="26" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D26" s="4" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="27" spans="2:7">
+    <row r="27" spans="2:7" x14ac:dyDescent="0.25">
       <c r="D27" s="4" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="34" spans="2:2">
+    <row r="34" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B34" s="12"/>
     </row>
   </sheetData>
@@ -6697,7 +6697,7 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{124CE633-E2C2-45EB-9187-AAB4045A946D}">
   <dimension ref="B1:G34"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="1"/>
     <col min="2" max="2" width="36" style="1" customWidth="1"/>
@@ -6709,36 +6709,36 @@
     <col min="8" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:7" ht="30" customHeight="1"/>
-    <row r="2" spans="2:7" ht="25.5" customHeight="1">
+    <row r="1" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="2:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="5" t="s">
         <v>85</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="F2" s="13" t="s">
+      <c r="F2" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="13"/>
-    </row>
-    <row r="3" spans="2:7" ht="25.5" customHeight="1">
+      <c r="G2" s="18"/>
+    </row>
+    <row r="3" spans="2:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="3">
         <v>520000</v>
       </c>
       <c r="D3" s="3">
         <v>920000</v>
       </c>
-      <c r="F3" s="13"/>
-      <c r="G3" s="13"/>
-    </row>
-    <row r="4" spans="2:7" ht="6" customHeight="1">
+      <c r="F3" s="18"/>
+      <c r="G3" s="18"/>
+    </row>
+    <row r="4" spans="2:7" ht="6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="4"/>
       <c r="D4" s="4"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
     </row>
-    <row r="5" spans="2:7">
+    <row r="5" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B5" s="4" t="s">
         <v>80</v>
       </c>
@@ -6752,7 +6752,7 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="6" spans="2:7">
+    <row r="6" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B6" s="4" t="s">
         <v>64</v>
       </c>
@@ -6766,7 +6766,7 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="7" spans="2:7">
+    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B7" s="4" t="s">
         <v>65</v>
       </c>
@@ -6780,7 +6780,7 @@
         <v>350000</v>
       </c>
     </row>
-    <row r="8" spans="2:7">
+    <row r="8" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B8" s="4" t="s">
         <v>4</v>
       </c>
@@ -6794,50 +6794,50 @@
         <v>50000</v>
       </c>
     </row>
-    <row r="9" spans="2:7">
+    <row r="9" spans="2:7" x14ac:dyDescent="0.25">
       <c r="D9" s="4" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="10" spans="2:7">
+    <row r="10" spans="2:7" x14ac:dyDescent="0.25">
       <c r="D10" s="4" t="s">
         <v>4</v>
       </c>
       <c r="F10" s="10"/>
       <c r="G10" s="11"/>
     </row>
-    <row r="12" spans="2:7">
+    <row r="12" spans="2:7" x14ac:dyDescent="0.25">
       <c r="D12" s="10"/>
     </row>
-    <row r="14" spans="2:7" ht="26.25" customHeight="1">
+    <row r="14" spans="2:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="5" t="s">
         <v>86</v>
       </c>
       <c r="D14" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="F14" s="14" t="s">
+      <c r="F14" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="G14" s="13"/>
-    </row>
-    <row r="15" spans="2:7" ht="25.5" customHeight="1">
+      <c r="G14" s="18"/>
+    </row>
+    <row r="15" spans="2:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="3">
         <v>1600000</v>
       </c>
       <c r="D15" s="3">
         <v>4800000</v>
       </c>
-      <c r="F15" s="13"/>
-      <c r="G15" s="13"/>
-    </row>
-    <row r="16" spans="2:7" ht="6.75" customHeight="1">
+      <c r="F15" s="18"/>
+      <c r="G15" s="18"/>
+    </row>
+    <row r="16" spans="2:7" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="4"/>
       <c r="D16" s="4"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
     </row>
-    <row r="17" spans="2:7">
+    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B17" s="4" t="s">
         <v>81</v>
       </c>
@@ -6851,7 +6851,7 @@
         <v>-50000</v>
       </c>
     </row>
-    <row r="18" spans="2:7">
+    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B18" s="4" t="s">
         <v>64</v>
       </c>
@@ -6866,7 +6866,7 @@
         <v>-50000 &amp; -25000</v>
       </c>
     </row>
-    <row r="19" spans="2:7">
+    <row r="19" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B19" s="4" t="s">
         <v>57</v>
       </c>
@@ -6881,7 +6881,7 @@
         <v>-50% All Type</v>
       </c>
     </row>
-    <row r="20" spans="2:7">
+    <row r="20" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B20" s="4" t="s">
         <v>69</v>
       </c>
@@ -6889,7 +6889,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="21" spans="2:7">
+    <row r="21" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B21" s="4" t="s">
         <v>58</v>
       </c>
@@ -6897,7 +6897,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="22" spans="2:7">
+    <row r="22" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B22" s="4" t="s">
         <v>66</v>
       </c>
@@ -6905,7 +6905,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="23" spans="2:7">
+    <row r="23" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B23" s="4" t="s">
         <v>4</v>
       </c>
@@ -6913,14 +6913,14 @@
         <v>66</v>
       </c>
     </row>
-    <row r="24" spans="2:7">
+    <row r="24" spans="2:7" x14ac:dyDescent="0.25">
       <c r="D24" s="4" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="25" spans="2:7" ht="15.75" customHeight="1"/>
-    <row r="26" spans="2:7" ht="15.75" customHeight="1"/>
-    <row r="34" spans="2:2">
+    <row r="25" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="26" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="34" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B34" s="12"/>
     </row>
   </sheetData>

</xml_diff>